<commit_message>
Corrige data do AG10: 25/09/2026 (não 18/09)
O usuário confirmou, olhando o arquivo local, que o AG10 (10C1/10C2)
não é mais no último dia de P1 (18/09) — a escola remarcou para
25/09/2026 (sexta da semana 8, já dentro do pool de P2). A janela de
P1 (24/08-18/09) em si não muda com este ajuste, só a data do AG10.

- SIMULADOS: AG10 (10C1, 10C2) muda de (7,5) para (8,5).
- Regenera as 3 propostas; verificador passa em tudo (só os avisos
  de sempre em tempos 7-11). Proposta 3 fechou com os cinco limites
  de cessão estritos, sem exceção (pior caso 10,7%, igual a antes).
- Regenera relatórios de exportação (tempos cedidos, tabela por turma).
- Atualiza referencia/estado_2sem_2026.md com a nova data e o
  histórico do ajuste (não a skill genérica).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Proposta_1_Calendario_Provas_2026_2SEM.xlsx
+++ b/Horario desenvolvido/Proposta_1_Calendario_Provas_2026_2SEM.xlsx
@@ -12008,19 +12008,19 @@
         </is>
       </c>
       <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>GL - EFr-Car-Swa
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>DaF - Eth-EFr-Swa
+4º e 5º tempos</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Geo - Mlo
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>Mat - BrSa/FBri
-4º e 5º tempos</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="n"/>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
       <c r="M12" s="15" t="n"/>
@@ -12084,11 +12084,16 @@
         </is>
       </c>
       <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>GL - EFr-Car-Swa
+2º e 3º tempos</t>
+        </is>
+      </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Hist - ALu
-2º e 3º tempos</t>
+          <t>Fis - VSi
+1º e 2º tempos</t>
         </is>
       </c>
       <c r="I15" s="11" t="n"/>
@@ -12157,16 +12162,11 @@
 6º e 7º tempos</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>DaF - Eth-EFr-Swa
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="G18" s="11" t="n"/>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>Geo - Mlo
-4º e 5º tempos</t>
+          <t>LP/LIT/RED - BPad/MFo/SMo
+1º ao 3º tempos</t>
         </is>
       </c>
       <c r="I18" s="350" t="n"/>
@@ -12237,24 +12237,19 @@
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>LP/LIT/RED - BPad/MFo/SMo
-1º ao 3º tempos</t>
+          <t>Mat - BrSa/FBri
+2º e 3º tempos</t>
         </is>
       </c>
       <c r="F21" s="62" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>Fis - VSi
-1º e 2º tempos</t>
-        </is>
-      </c>
-      <c r="I21" s="11" t="inlineStr">
-        <is>
-          <t>AG10
-2º ao 7º tempos</t>
-        </is>
-      </c>
+          <t>Hist - ALu
+2º e 3º tempos</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="n"/>
       <c r="J21" s="183" t="n"/>
       <c r="L21" s="80" t="inlineStr">
         <is>
@@ -12319,19 +12314,19 @@
       </c>
       <c r="E24" s="283" t="inlineStr">
         <is>
-          <t>Qui - CAl
-4º e 5º tempos</t>
+          <t>LP/LIT/RED - BPad/MFo/SMo
+1º ao 3º tempos</t>
         </is>
       </c>
       <c r="F24" s="283" t="n"/>
       <c r="G24" s="79" t="n"/>
-      <c r="H24" s="283" t="inlineStr">
-        <is>
-          <t>Geo - Mlo
-4º e 5º tempos</t>
-        </is>
-      </c>
-      <c r="I24" s="78" t="n"/>
+      <c r="H24" s="283" t="n"/>
+      <c r="I24" s="78" t="inlineStr">
+        <is>
+          <t>AG10
+2º ao 7º tempos</t>
+        </is>
+      </c>
       <c r="J24" s="265" t="n"/>
       <c r="L24" s="318" t="inlineStr">
         <is>
@@ -12399,16 +12394,16 @@
       </c>
       <c r="E27" s="78" t="inlineStr">
         <is>
-          <t>LP/LIT/RED - BPad/MFo/SMo
-1º ao 3º tempos</t>
+          <t>Mat - BrSa/FBri
+1º e 2º tempos</t>
         </is>
       </c>
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="283" t="n"/>
       <c r="H27" s="283" t="inlineStr">
         <is>
-          <t>Fis - VSi
-1º e 2º tempos</t>
+          <t>Hist - ALu
+2º e 3º tempos</t>
         </is>
       </c>
       <c r="I27" s="283" t="n"/>
@@ -12477,13 +12472,13 @@
         <f>B30+4</f>
         <v/>
       </c>
-      <c r="E30" s="283" t="n"/>
-      <c r="F30" s="283" t="inlineStr">
-        <is>
-          <t>Bio - Lza
-10º e 11º tempos</t>
-        </is>
-      </c>
+      <c r="E30" s="283" t="inlineStr">
+        <is>
+          <t>Fis - VSi
+4º e 5º tempos</t>
+        </is>
+      </c>
+      <c r="F30" s="283" t="n"/>
       <c r="G30" s="283" t="n"/>
       <c r="H30" s="283" t="n"/>
       <c r="I30" s="283" t="n"/>
@@ -12653,14 +12648,19 @@
         <v/>
       </c>
       <c r="E36" s="283" t="n"/>
-      <c r="F36" s="283" t="n"/>
-      <c r="G36" s="283" t="inlineStr">
-        <is>
-          <t>GL - EFr-Car-Swa
+      <c r="F36" s="283" t="inlineStr">
+        <is>
+          <t>Bio - Lza
+10º e 11º tempos</t>
+        </is>
+      </c>
+      <c r="G36" s="283" t="n"/>
+      <c r="H36" s="283" t="inlineStr">
+        <is>
+          <t>Ing - APa
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="H36" s="283" t="n"/>
       <c r="I36" s="283" t="n"/>
       <c r="J36" s="265" t="n"/>
       <c r="L36" s="81" t="inlineStr">
@@ -12730,14 +12730,14 @@
       <c r="F39" s="283" t="n"/>
       <c r="G39" s="283" t="inlineStr">
         <is>
-          <t>Fil - LAn
-1º tempo</t>
+          <t>GL - EFr-Car-Swa
+2º e 3º tempos</t>
         </is>
       </c>
       <c r="H39" s="283" t="inlineStr">
         <is>
-          <t>Ing - APa
-2º e 3º tempos</t>
+          <t>Geo - Mlo
+4º e 5º tempos</t>
         </is>
       </c>
       <c r="I39" s="283" t="n"/>
@@ -12787,13 +12787,13 @@
       </c>
       <c r="E42" s="283" t="n"/>
       <c r="F42" s="283" t="n"/>
-      <c r="G42" s="283" t="n"/>
-      <c r="H42" s="283" t="inlineStr">
-        <is>
-          <t>Mat - BrSa/FBri
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="G42" s="283" t="inlineStr">
+        <is>
+          <t>Fil - LAn
+1º tempo</t>
+        </is>
+      </c>
+      <c r="H42" s="283" t="n"/>
       <c r="I42" s="283" t="inlineStr">
         <is>
           <t>Soc - Kle
@@ -12852,7 +12852,12 @@
         <f>B45+4</f>
         <v/>
       </c>
-      <c r="E45" s="283" t="n"/>
+      <c r="E45" s="283" t="inlineStr">
+        <is>
+          <t>Qui - CAl
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="F45" s="283" t="n"/>
       <c r="G45" s="283" t="inlineStr">
         <is>
@@ -12860,12 +12865,7 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="H45" s="283" t="inlineStr">
-        <is>
-          <t>Hist - ALu
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="H45" s="283" t="n"/>
       <c r="I45" s="358" t="inlineStr">
         <is>
           <t>2CH
@@ -13689,19 +13689,19 @@
         </is>
       </c>
       <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>GL - EFr-Car-Swa
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>DaF - Eth-EFr-Swa
+4º e 5º tempos</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Geo - Mlo
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>Mat - BrSa/FBri
-4º e 5º tempos</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="n"/>
       <c r="J12" s="183" t="n"/>
       <c r="L12" s="15" t="n"/>
       <c r="M12" s="15" t="n"/>
@@ -13765,11 +13765,16 @@
 4º e 5º tempos</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n"/>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>GL - EFr-Car-Swa
+2º e 3º tempos</t>
+        </is>
+      </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Hist - ALu
-2º e 3º tempos</t>
+          <t>Fis - VSi
+1º e 2º tempos</t>
         </is>
       </c>
       <c r="I15" s="11" t="n"/>
@@ -13838,16 +13843,11 @@
 6º e 7º tempos</t>
         </is>
       </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>DaF - Eth-EFr-Swa
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="G18" s="11" t="n"/>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>Geo - Mlo
-4º e 5º tempos</t>
+          <t>LP/LIT/RED - BPad/MFo/SMo
+1º ao 3º tempos</t>
         </is>
       </c>
       <c r="I18" s="350" t="n"/>
@@ -13918,24 +13918,19 @@
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>LP/LIT/RED - BPad/MFo/SMo
-1º ao 3º tempos</t>
+          <t>Mat - BrSa/FBri
+2º e 3º tempos</t>
         </is>
       </c>
       <c r="F21" s="62" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>Fis - VSi
-1º e 2º tempos</t>
-        </is>
-      </c>
-      <c r="I21" s="11" t="inlineStr">
-        <is>
-          <t>AG10
-2º ao 7º tempos</t>
-        </is>
-      </c>
+          <t>Hist - ALu
+2º e 3º tempos</t>
+        </is>
+      </c>
+      <c r="I21" s="11" t="n"/>
       <c r="J21" s="183" t="n"/>
       <c r="L21" s="80" t="inlineStr">
         <is>
@@ -14000,19 +13995,19 @@
       </c>
       <c r="E24" s="283" t="inlineStr">
         <is>
-          <t>Qui - CAl
-4º e 5º tempos</t>
+          <t>LP/LIT/RED - BPad/MFo/SMo
+1º ao 3º tempos</t>
         </is>
       </c>
       <c r="F24" s="283" t="n"/>
       <c r="G24" s="79" t="n"/>
-      <c r="H24" s="283" t="inlineStr">
-        <is>
-          <t>Geo - Mlo
-4º e 5º tempos</t>
-        </is>
-      </c>
-      <c r="I24" s="78" t="n"/>
+      <c r="H24" s="283" t="n"/>
+      <c r="I24" s="78" t="inlineStr">
+        <is>
+          <t>AG10
+2º ao 7º tempos</t>
+        </is>
+      </c>
       <c r="J24" s="265" t="n"/>
       <c r="L24" s="318" t="inlineStr">
         <is>
@@ -14080,16 +14075,16 @@
       </c>
       <c r="E27" s="78" t="inlineStr">
         <is>
-          <t>LP/LIT/RED - BPad/MFo/SMo
-1º ao 3º tempos</t>
+          <t>Mat - BrSa/FBri
+1º e 2º tempos</t>
         </is>
       </c>
       <c r="F27" s="283" t="n"/>
       <c r="G27" s="283" t="n"/>
       <c r="H27" s="283" t="inlineStr">
         <is>
-          <t>Fis - VSi
-1º e 2º tempos</t>
+          <t>Hist - ALu
+2º e 3º tempos</t>
         </is>
       </c>
       <c r="I27" s="283" t="n"/>
@@ -14158,13 +14153,13 @@
         <f>B30+4</f>
         <v/>
       </c>
-      <c r="E30" s="283" t="n"/>
-      <c r="F30" s="283" t="inlineStr">
-        <is>
-          <t>Bio - Lza
-10º e 11º tempos</t>
-        </is>
-      </c>
+      <c r="E30" s="283" t="inlineStr">
+        <is>
+          <t>Fis - VSi
+4º e 5º tempos</t>
+        </is>
+      </c>
+      <c r="F30" s="283" t="n"/>
       <c r="G30" s="283" t="inlineStr">
         <is>
           <t>Ing - Vir
@@ -14339,13 +14334,13 @@
         <v/>
       </c>
       <c r="E36" s="283" t="n"/>
-      <c r="F36" s="283" t="n"/>
-      <c r="G36" s="283" t="inlineStr">
-        <is>
-          <t>GL - EFr-Car-Swa
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="F36" s="283" t="inlineStr">
+        <is>
+          <t>Bio - Lza
+10º e 11º tempos</t>
+        </is>
+      </c>
+      <c r="G36" s="283" t="n"/>
       <c r="H36" s="283" t="n"/>
       <c r="I36" s="283" t="n"/>
       <c r="J36" s="265" t="n"/>
@@ -14416,11 +14411,16 @@
       <c r="F39" s="283" t="n"/>
       <c r="G39" s="283" t="inlineStr">
         <is>
-          <t>Fil - LAn
-1º tempo</t>
-        </is>
-      </c>
-      <c r="H39" s="283" t="n"/>
+          <t>GL - EFr-Car-Swa
+2º e 3º tempos</t>
+        </is>
+      </c>
+      <c r="H39" s="283" t="inlineStr">
+        <is>
+          <t>Geo - Mlo
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="I39" s="283" t="n"/>
       <c r="J39" s="265" t="n"/>
     </row>
@@ -14468,13 +14468,13 @@
       </c>
       <c r="E42" s="283" t="n"/>
       <c r="F42" s="283" t="n"/>
-      <c r="G42" s="283" t="n"/>
-      <c r="H42" s="283" t="inlineStr">
-        <is>
-          <t>Mat - BrSa/FBri
-4º e 5º tempos</t>
-        </is>
-      </c>
+      <c r="G42" s="283" t="inlineStr">
+        <is>
+          <t>Fil - LAn
+1º tempo</t>
+        </is>
+      </c>
+      <c r="H42" s="283" t="n"/>
       <c r="I42" s="283" t="inlineStr">
         <is>
           <t>Soc - Kle
@@ -14533,7 +14533,12 @@
         <f>B45+4</f>
         <v/>
       </c>
-      <c r="E45" s="283" t="n"/>
+      <c r="E45" s="283" t="inlineStr">
+        <is>
+          <t>Qui - CAl
+4º e 5º tempos</t>
+        </is>
+      </c>
       <c r="F45" s="283" t="n"/>
       <c r="G45" s="283" t="inlineStr">
         <is>
@@ -14541,12 +14546,7 @@
 2º e 3º tempos</t>
         </is>
       </c>
-      <c r="H45" s="283" t="inlineStr">
-        <is>
-          <t>Hist - ALu
-2º e 3º tempos</t>
-        </is>
-      </c>
+      <c r="H45" s="283" t="n"/>
       <c r="I45" s="358" t="inlineStr">
         <is>
           <t>2CH

</xml_diff>